<commit_message>
New app added + New Member Onboarding instructions
</commit_message>
<xml_diff>
--- a/src/apps/orangehrms/data/testdata.xlsx
+++ b/src/apps/orangehrms/data/testdata.xlsx
@@ -6,13 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="LoginData" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="ClaimData" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="DashboardLinksData" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="QuickLaunchLinksData" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="89">
   <si>
     <t>testCaseId</t>
   </si>
@@ -120,6 +122,165 @@
   </si>
   <si>
     <t>Airfare and local transport for client site visit</t>
+  </si>
+  <si>
+    <t>linkName</t>
+  </si>
+  <si>
+    <t>expectedUrlFragment</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_01</t>
+  </si>
+  <si>
+    <t>admin/viewSystemUsers</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_02</t>
+  </si>
+  <si>
+    <t>PIM</t>
+  </si>
+  <si>
+    <t>pim/viewEmployeeList</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_03</t>
+  </si>
+  <si>
+    <t>Leave</t>
+  </si>
+  <si>
+    <t>leave/viewLeaveList</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_04</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>time/viewEmployeeTimesheet</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_05</t>
+  </si>
+  <si>
+    <t>Recruitment</t>
+  </si>
+  <si>
+    <t>recruitment/viewCandidates</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_06</t>
+  </si>
+  <si>
+    <t>My Info</t>
+  </si>
+  <si>
+    <t>pim/viewPersonalDetails</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_07</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>performance/searchEvaluatePerformanceReview</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_08</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>dashboard/index</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_09</t>
+  </si>
+  <si>
+    <t>Directory</t>
+  </si>
+  <si>
+    <t>directory/viewDirectory</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_10</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>maintenance/purgeEmployee</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_11</t>
+  </si>
+  <si>
+    <t>Claim</t>
+  </si>
+  <si>
+    <t>claim/viewAssignClaim</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_12</t>
+  </si>
+  <si>
+    <t>Buzz</t>
+  </si>
+  <si>
+    <t>buzz/viewBuzz</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_01</t>
+  </si>
+  <si>
+    <t>Assign Leave</t>
+  </si>
+  <si>
+    <t>leave/assignLeave</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_02</t>
+  </si>
+  <si>
+    <t>Leave List</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_03</t>
+  </si>
+  <si>
+    <t>Timesheets</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_04</t>
+  </si>
+  <si>
+    <t>Apply Leave</t>
+  </si>
+  <si>
+    <t>leave/applyLeave</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_05</t>
+  </si>
+  <si>
+    <t>My Leave</t>
+  </si>
+  <si>
+    <t>leave/viewMyLeaveList</t>
+  </si>
+  <si>
+    <t>TC_QUICKLAUNCH_06</t>
+  </si>
+  <si>
+    <t>My Timesheet</t>
+  </si>
+  <si>
+    <t>time/viewMyTimesheet</t>
   </si>
 </sst>
 </file>
@@ -736,4 +897,318 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>